<commit_message>
updated files and paxbox measurement
</commit_message>
<xml_diff>
--- a/Antonio-Feed/__FeedPartsInventory.xlsx
+++ b/Antonio-Feed/__FeedPartsInventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pollak/Documents/GitHub/Front-Page/Antonio-Feed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{510F6DBD-23CF-494F-A1A7-43D649DD396E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67215C1C-49E5-3A45-A12F-D400789CF140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-100000" yWindow="600" windowWidth="34200" windowHeight="19940" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-53560" yWindow="2120" windowWidth="34200" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts At ATA" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1287" uniqueCount="452">
   <si>
     <t>Antenna Inventory</t>
   </si>
@@ -1254,9 +1254,6 @@
     <t>X=0.12 Y=0.03 Z=0.09</t>
   </si>
   <si>
-    <t>QRFH</t>
-  </si>
-  <si>
     <t>2064Z / 2287Z</t>
   </si>
   <si>
@@ -1399,6 +1396,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>LAB1</t>
   </si>
 </sst>
 </file>
@@ -1515,7 +1515,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="24">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1646,12 +1646,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FFFF9900"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1995,7 +1989,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2213,11 +2207,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2235,6 +2224,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2253,6 +2246,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2491,25 +2488,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="122"/>
-      <c r="I1" s="123"/>
-      <c r="J1" s="123"/>
-      <c r="K1" s="122"/>
-      <c r="L1" s="123"/>
-      <c r="M1" s="123"/>
-      <c r="N1" s="123"/>
-      <c r="O1" s="123"/>
-      <c r="P1" s="123"/>
-      <c r="Q1" s="123"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
     </row>
     <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -2587,7 +2584,7 @@
         <v>20</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>225</v>
@@ -2948,7 +2945,7 @@
         <v>56</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>21</v>
@@ -3499,7 +3496,7 @@
         <v>4G</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>97</v>
@@ -3821,28 +3818,28 @@
       <c r="A58" s="3"/>
     </row>
     <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="124"/>
-      <c r="B59" s="119"/>
-      <c r="C59" s="119"/>
+      <c r="A59" s="121"/>
+      <c r="B59" s="116"/>
+      <c r="C59" s="116"/>
     </row>
     <row r="60" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="7"/>
     </row>
     <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="118"/>
-      <c r="B61" s="119"/>
-      <c r="C61" s="118"/>
-      <c r="D61" s="119"/>
-      <c r="E61" s="119"/>
-      <c r="F61" s="119"/>
+      <c r="A61" s="115"/>
+      <c r="B61" s="116"/>
+      <c r="C61" s="115"/>
+      <c r="D61" s="116"/>
+      <c r="E61" s="116"/>
+      <c r="F61" s="116"/>
     </row>
     <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="118"/>
-      <c r="B62" s="119"/>
-      <c r="C62" s="118"/>
-      <c r="D62" s="119"/>
-      <c r="E62" s="119"/>
-      <c r="F62" s="119"/>
+      <c r="A62" s="115"/>
+      <c r="B62" s="116"/>
+      <c r="C62" s="115"/>
+      <c r="D62" s="116"/>
+      <c r="E62" s="116"/>
+      <c r="F62" s="116"/>
     </row>
     <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4819,20 +4816,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="122" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="115"/>
-      <c r="C1" s="116" t="s">
+      <c r="B1" s="123"/>
+      <c r="C1" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
+      <c r="H1" s="114"/>
+      <c r="I1" s="114"/>
+      <c r="J1" s="114"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
@@ -4874,7 +4871,7 @@
         <v>281</v>
       </c>
       <c r="M2" s="56" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -5036,39 +5033,25 @@
         <v>5C4-005</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="J7" s="19" t="s">
-        <v>131</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
       <c r="K7" s="43" t="s">
         <v>319</v>
       </c>
       <c r="L7" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M7" s="98"/>
+      <c r="M7" s="19" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="str">
@@ -5193,37 +5176,23 @@
         <v>5C4-009</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>413</v>
-      </c>
-      <c r="C11" s="38" t="s">
+        <v>412</v>
+      </c>
+      <c r="C11" s="38"/>
+      <c r="D11" s="130"/>
+      <c r="E11" s="130"/>
+      <c r="F11" s="130"/>
+      <c r="G11" s="130"/>
+      <c r="H11" s="130"/>
+      <c r="I11" s="130"/>
+      <c r="J11" s="130"/>
+      <c r="K11" s="38" t="s">
         <v>403</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="I11" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="J11" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="K11" s="38" t="s">
-        <v>404</v>
-      </c>
       <c r="L11" s="38"/>
-      <c r="M11" s="98"/>
+      <c r="M11" s="38" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="12" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="str">
@@ -5689,7 +5658,7 @@
         <v>25</v>
       </c>
       <c r="K23" s="80" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="L23" s="12"/>
       <c r="M23" s="100">
@@ -5728,7 +5697,7 @@
         <v>25</v>
       </c>
       <c r="K24" s="80" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L24" s="38"/>
       <c r="M24" s="100">
@@ -5767,7 +5736,7 @@
         <v>25</v>
       </c>
       <c r="K25" s="80" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L25" s="38"/>
       <c r="M25" s="100">
@@ -5776,7 +5745,7 @@
     </row>
     <row r="26" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B26" s="86" t="s">
         <v>157</v>
@@ -5806,7 +5775,7 @@
         <v>25</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="L26" s="38"/>
       <c r="M26" s="100">
@@ -5815,7 +5784,7 @@
     </row>
     <row r="27" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B27" s="86" t="s">
         <v>232</v>
@@ -5845,7 +5814,7 @@
         <v>25</v>
       </c>
       <c r="K27" s="38" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L27" s="38"/>
       <c r="M27" s="100">
@@ -5854,10 +5823,10 @@
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B28" s="107" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C28" s="108"/>
       <c r="D28" s="109" t="s">
@@ -5881,10 +5850,10 @@
     </row>
     <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="106" t="s">
-        <v>433</v>
-      </c>
-      <c r="B29" s="113" t="s">
-        <v>385</v>
+        <v>432</v>
+      </c>
+      <c r="B29" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C29" s="54"/>
       <c r="D29" s="112"/>
@@ -5900,10 +5869,10 @@
     </row>
     <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="106" t="s">
-        <v>434</v>
-      </c>
-      <c r="B30" s="113" t="s">
-        <v>385</v>
+        <v>433</v>
+      </c>
+      <c r="B30" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C30" s="54"/>
       <c r="D30" s="112"/>
@@ -5919,10 +5888,10 @@
     </row>
     <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="106" t="s">
-        <v>435</v>
-      </c>
-      <c r="B31" s="113" t="s">
-        <v>385</v>
+        <v>434</v>
+      </c>
+      <c r="B31" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C31" s="54"/>
       <c r="D31" s="112"/>
@@ -5938,10 +5907,10 @@
     </row>
     <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="106" t="s">
-        <v>436</v>
-      </c>
-      <c r="B32" s="113" t="s">
-        <v>385</v>
+        <v>435</v>
+      </c>
+      <c r="B32" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C32" s="54"/>
       <c r="D32" s="112"/>
@@ -5957,10 +5926,10 @@
     </row>
     <row r="33" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="106" t="s">
-        <v>437</v>
-      </c>
-      <c r="B33" s="113" t="s">
-        <v>385</v>
+        <v>436</v>
+      </c>
+      <c r="B33" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C33" s="54"/>
       <c r="D33" s="112"/>
@@ -5976,10 +5945,10 @@
     </row>
     <row r="34" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="106" t="s">
-        <v>438</v>
-      </c>
-      <c r="B34" s="113" t="s">
-        <v>385</v>
+        <v>437</v>
+      </c>
+      <c r="B34" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C34" s="54"/>
       <c r="D34" s="112"/>
@@ -5995,10 +5964,10 @@
     </row>
     <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="106" t="s">
-        <v>439</v>
-      </c>
-      <c r="B35" s="113" t="s">
-        <v>385</v>
+        <v>438</v>
+      </c>
+      <c r="B35" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C35" s="54"/>
       <c r="D35" s="112"/>
@@ -6014,10 +5983,10 @@
     </row>
     <row r="36" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="106" t="s">
-        <v>440</v>
-      </c>
-      <c r="B36" s="113" t="s">
-        <v>385</v>
+        <v>439</v>
+      </c>
+      <c r="B36" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C36" s="54"/>
       <c r="D36" s="112"/>
@@ -6033,10 +6002,10 @@
     </row>
     <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="106" t="s">
-        <v>441</v>
-      </c>
-      <c r="B37" s="113" t="s">
-        <v>385</v>
+        <v>440</v>
+      </c>
+      <c r="B37" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C37" s="54"/>
       <c r="D37" s="112"/>
@@ -6052,10 +6021,10 @@
     </row>
     <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="106" t="s">
-        <v>442</v>
-      </c>
-      <c r="B38" s="113" t="s">
-        <v>385</v>
+        <v>441</v>
+      </c>
+      <c r="B38" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C38" s="54"/>
       <c r="D38" s="112"/>
@@ -6071,10 +6040,10 @@
     </row>
     <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="106" t="s">
-        <v>443</v>
-      </c>
-      <c r="B39" s="113" t="s">
-        <v>385</v>
+        <v>442</v>
+      </c>
+      <c r="B39" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C39" s="54"/>
       <c r="D39" s="112"/>
@@ -6090,10 +6059,10 @@
     </row>
     <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="106" t="s">
-        <v>444</v>
-      </c>
-      <c r="B40" s="113" t="s">
-        <v>385</v>
+        <v>443</v>
+      </c>
+      <c r="B40" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C40" s="54"/>
       <c r="D40" s="112"/>
@@ -6109,10 +6078,10 @@
     </row>
     <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="106" t="s">
-        <v>445</v>
-      </c>
-      <c r="B41" s="113" t="s">
-        <v>385</v>
+        <v>444</v>
+      </c>
+      <c r="B41" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C41" s="54"/>
       <c r="D41" s="112"/>
@@ -6128,10 +6097,10 @@
     </row>
     <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="106" t="s">
-        <v>446</v>
-      </c>
-      <c r="B42" s="113" t="s">
-        <v>385</v>
+        <v>445</v>
+      </c>
+      <c r="B42" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C42" s="54"/>
       <c r="D42" s="112"/>
@@ -6147,10 +6116,10 @@
     </row>
     <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="106" t="s">
-        <v>447</v>
-      </c>
-      <c r="B43" s="113" t="s">
-        <v>385</v>
+        <v>446</v>
+      </c>
+      <c r="B43" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C43" s="54"/>
       <c r="D43" s="112"/>
@@ -6166,10 +6135,10 @@
     </row>
     <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="106" t="s">
-        <v>448</v>
-      </c>
-      <c r="B44" s="113" t="s">
-        <v>385</v>
+        <v>447</v>
+      </c>
+      <c r="B44" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C44" s="54"/>
       <c r="D44" s="112"/>
@@ -6185,10 +6154,10 @@
     </row>
     <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="106" t="s">
-        <v>449</v>
-      </c>
-      <c r="B45" s="113" t="s">
-        <v>385</v>
+        <v>448</v>
+      </c>
+      <c r="B45" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C45" s="54"/>
       <c r="D45" s="112"/>
@@ -6204,10 +6173,10 @@
     </row>
     <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="106" t="s">
-        <v>450</v>
-      </c>
-      <c r="B46" s="113" t="s">
-        <v>385</v>
+        <v>449</v>
+      </c>
+      <c r="B46" s="131" t="s">
+        <v>451</v>
       </c>
       <c r="C46" s="54"/>
       <c r="D46" s="112"/>
@@ -6242,14 +6211,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="113" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
       <c r="G1" s="61"/>
       <c r="H1" s="61"/>
       <c r="I1" s="61"/>
@@ -6558,7 +6527,7 @@
         <v>360</v>
       </c>
       <c r="F14" s="62" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -6871,36 +6840,34 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="104" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B29" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>428</v>
+      </c>
+      <c r="E29" s="105" t="s">
         <v>430</v>
       </c>
-      <c r="C29" s="33" t="s">
-        <v>429</v>
-      </c>
-      <c r="E29" s="105" t="s">
+      <c r="G29" s="33" t="s">
         <v>431</v>
-      </c>
-      <c r="G29" s="33" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="104" t="s">
+        <v>425</v>
+      </c>
+      <c r="B30" s="33" t="s">
         <v>426</v>
       </c>
-      <c r="B30" s="33" t="s">
+      <c r="C30" s="33" t="s">
         <v>427</v>
       </c>
-      <c r="C30" s="33" t="s">
-        <v>428</v>
-      </c>
-      <c r="E30" s="105" t="s">
+      <c r="E30" s="105"/>
+      <c r="G30" s="33" t="s">
         <v>431</v>
-      </c>
-      <c r="G30" s="33" t="s">
-        <v>432</v>
       </c>
     </row>
   </sheetData>
@@ -6924,20 +6891,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="124" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="125" t="s">
+      <c r="B1" s="125"/>
+      <c r="C1" s="124" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="125"/>
     </row>
     <row r="2" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
@@ -7124,7 +7091,7 @@
         <v>243</v>
       </c>
       <c r="B11" s="59" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C11" s="32" t="s">
         <v>261</v>
@@ -7336,7 +7303,7 @@
         <v>250</v>
       </c>
       <c r="B22" s="41" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C22" s="36" t="s">
         <v>401</v>
@@ -7401,14 +7368,14 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="28" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B26" s="41" t="s">
         <v>157</v>
       </c>
       <c r="C26" s="36"/>
       <c r="D26" s="32" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E26" s="32"/>
       <c r="F26" s="32"/>
@@ -7419,7 +7386,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="28" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B27" s="41" t="s">
         <v>232</v>
@@ -7435,16 +7402,16 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="28" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B28" s="92" t="s">
         <v>126</v>
       </c>
       <c r="C28" s="36" t="s">
+        <v>421</v>
+      </c>
+      <c r="D28" s="36" t="s">
         <v>422</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>423</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -7495,21 +7462,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>297</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
       <c r="D1" s="81"/>
-      <c r="E1" s="122" t="s">
+      <c r="E1" s="119" t="s">
         <v>397</v>
       </c>
-      <c r="F1" s="122"/>
-      <c r="G1" s="122"/>
-      <c r="H1" s="130" t="s">
-        <v>410</v>
-      </c>
-      <c r="I1" s="130"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="129" t="s">
+        <v>409</v>
+      </c>
+      <c r="I1" s="129"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="82" t="s">
@@ -7534,7 +7501,7 @@
         <v>400</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -7613,7 +7580,7 @@
         <v>25</v>
       </c>
       <c r="H5" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -7665,7 +7632,7 @@
         <v>25</v>
       </c>
       <c r="H7" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -7719,7 +7686,7 @@
         <v>25</v>
       </c>
       <c r="H9" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -7746,7 +7713,7 @@
         <v>25</v>
       </c>
       <c r="H10" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -7798,7 +7765,7 @@
         <v>25</v>
       </c>
       <c r="H12" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -7825,7 +7792,7 @@
         <v>25</v>
       </c>
       <c r="H13" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -7852,7 +7819,7 @@
         <v>25</v>
       </c>
       <c r="H14" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -7879,7 +7846,7 @@
         <v>25</v>
       </c>
       <c r="H15" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -7931,7 +7898,7 @@
         <v>25</v>
       </c>
       <c r="H17" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -8008,7 +7975,7 @@
         <v>25</v>
       </c>
       <c r="H20" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -8035,7 +8002,7 @@
         <v>25</v>
       </c>
       <c r="H21" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -8062,7 +8029,7 @@
         <v>25</v>
       </c>
       <c r="H22" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -8089,7 +8056,7 @@
         <v>25</v>
       </c>
       <c r="H23" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -8116,7 +8083,7 @@
         <v>25</v>
       </c>
       <c r="H24" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -8143,7 +8110,7 @@
         <v>25</v>
       </c>
       <c r="H25" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -8170,7 +8137,7 @@
         <v>25</v>
       </c>
       <c r="H26" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -8302,7 +8269,7 @@
         <v>25</v>
       </c>
       <c r="H32" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -8329,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="H33" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -8433,7 +8400,7 @@
         <v>25</v>
       </c>
       <c r="H37" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -8510,7 +8477,7 @@
         <v>25</v>
       </c>
       <c r="H40" s="73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -8670,7 +8637,7 @@
       <c r="D4" s="69"/>
       <c r="E4" s="69"/>
       <c r="G4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">

</xml_diff>